<commit_message>
feat: integrate real tax monitoring workflows
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/tax_master_duplicate.xlsx
+++ b/backend/tests/fixtures/tax_master_duplicate.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,10 +448,15 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>deferred_tax_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>loss_carryforward</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>three_year_average_tax_burden</t>
         </is>
@@ -479,10 +484,15 @@
           <t>25%</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>9%</t>
         </is>
@@ -508,10 +518,15 @@
           <t>25%</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>9%</t>
         </is>

</xml_diff>